<commit_message>
adjust good moral certificate
</commit_message>
<xml_diff>
--- a/myapp/cert_templates/good-moral-form.xlsx
+++ b/myapp/cert_templates/good-moral-form.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\thesis_osa\myapp\cert_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A2E9447-8957-4B22-9D0E-627189A65B25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8398E4D-82B5-4D24-8E70-1ABCC6C9C08A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,6 +22,7 @@
     <definedName name="admission_date">inputs!$B$7</definedName>
     <definedName name="date_graduated">inputs!$B$8</definedName>
     <definedName name="osahead">inputs!$B$11</definedName>
+    <definedName name="osahead_title">inputs!$B$12</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">GMF!$H:$P</definedName>
     <definedName name="program">inputs!$B$3</definedName>
     <definedName name="purpose">inputs!$B$9</definedName>
@@ -29,7 +30,6 @@
     <definedName name="sex">inputs!$B$4</definedName>
     <definedName name="status">inputs!$B$5</definedName>
     <definedName name="student_name">inputs!$B$2</definedName>
-    <definedName name="title">inputs!$B$12</definedName>
     <definedName name="years_of_stay">inputs!$B$6</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -163,7 +163,7 @@
     <t>PRINCE JONE ARMAN JOHN MARS C. DELA CRUZ</t>
   </si>
   <si>
-    <t>title</t>
+    <t>osahead_title</t>
   </si>
 </sst>
 </file>
@@ -397,6 +397,36 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -407,36 +437,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -2168,15 +2168,15 @@
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
-      <c r="M2" s="21"/>
-      <c r="N2" s="21"/>
-      <c r="O2" s="21"/>
-      <c r="P2" s="21"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
+      <c r="O2" s="31"/>
+      <c r="P2" s="31"/>
     </row>
     <row r="3" spans="3:16" x14ac:dyDescent="0.25">
       <c r="D3" s="4"/>
@@ -2213,30 +2213,30 @@
       <c r="E5" s="9"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="22"/>
-      <c r="P5" s="22"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="32"/>
+      <c r="M5" s="32"/>
+      <c r="N5" s="32"/>
+      <c r="O5" s="32"/>
+      <c r="P5" s="32"/>
     </row>
     <row r="6" spans="3:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
-      <c r="M6" s="22"/>
-      <c r="N6" s="22"/>
-      <c r="O6" s="22"/>
-      <c r="P6" s="22"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="32"/>
+      <c r="M6" s="32"/>
+      <c r="N6" s="32"/>
+      <c r="O6" s="32"/>
+      <c r="P6" s="32"/>
     </row>
     <row r="7" spans="3:16" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D7" s="4" t="s">
@@ -2245,15 +2245,15 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
-      <c r="J7" s="24"/>
-      <c r="K7" s="24"/>
-      <c r="L7" s="24"/>
-      <c r="M7" s="24"/>
-      <c r="N7" s="24"/>
-      <c r="O7" s="24"/>
-      <c r="P7" s="24"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="34"/>
+      <c r="K7" s="34"/>
+      <c r="L7" s="34"/>
+      <c r="M7" s="34"/>
+      <c r="N7" s="34"/>
+      <c r="O7" s="34"/>
+      <c r="P7" s="34"/>
     </row>
     <row r="8" spans="3:16" x14ac:dyDescent="0.25">
       <c r="D8" s="4"/>
@@ -2268,15 +2268,15 @@
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="25"/>
-      <c r="J9" s="25"/>
-      <c r="K9" s="25"/>
-      <c r="L9" s="25"/>
-      <c r="M9" s="25"/>
-      <c r="N9" s="25"/>
-      <c r="O9" s="25"/>
-      <c r="P9" s="25"/>
+      <c r="H9" s="29"/>
+      <c r="I9" s="29"/>
+      <c r="J9" s="29"/>
+      <c r="K9" s="29"/>
+      <c r="L9" s="29"/>
+      <c r="M9" s="29"/>
+      <c r="N9" s="29"/>
+      <c r="O9" s="29"/>
+      <c r="P9" s="29"/>
     </row>
     <row r="10" spans="3:16" ht="2.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C10" s="4"/>
@@ -2317,13 +2317,13 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
-      <c r="K13" s="26" t="s">
+      <c r="K13" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="L13" s="26"/>
-      <c r="M13" s="26"/>
-      <c r="N13" s="26"/>
-      <c r="O13" s="26"/>
+      <c r="L13" s="21"/>
+      <c r="M13" s="21"/>
+      <c r="N13" s="21"/>
+      <c r="O13" s="21"/>
     </row>
     <row r="14" spans="3:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C14" s="4"/>
@@ -2338,13 +2338,13 @@
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
-      <c r="K15" s="27" t="s">
+      <c r="K15" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="L15" s="27"/>
-      <c r="M15" s="27"/>
-      <c r="N15" s="27"/>
-      <c r="O15" s="27"/>
+      <c r="L15" s="30"/>
+      <c r="M15" s="30"/>
+      <c r="N15" s="30"/>
+      <c r="O15" s="30"/>
     </row>
     <row r="16" spans="3:16" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C16" s="4"/>
@@ -2359,13 +2359,13 @@
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
-      <c r="K17" s="27" t="s">
+      <c r="K17" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="L17" s="27"/>
-      <c r="M17" s="27"/>
-      <c r="N17" s="27"/>
-      <c r="O17" s="27"/>
+      <c r="L17" s="30"/>
+      <c r="M17" s="30"/>
+      <c r="N17" s="30"/>
+      <c r="O17" s="30"/>
     </row>
     <row r="18" spans="3:15" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C18" s="4"/>
@@ -2375,11 +2375,11 @@
         <v>22</v>
       </c>
       <c r="G18" s="4"/>
-      <c r="K18" s="27"/>
-      <c r="L18" s="27"/>
-      <c r="M18" s="27"/>
-      <c r="N18" s="27"/>
-      <c r="O18" s="27"/>
+      <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
+      <c r="M18" s="30"/>
+      <c r="N18" s="30"/>
+      <c r="O18" s="30"/>
     </row>
     <row r="19" spans="3:15" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C19" s="4"/>
@@ -2387,13 +2387,13 @@
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
-      <c r="K19" s="28" t="s">
+      <c r="K19" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="L19" s="28"/>
-      <c r="M19" s="28"/>
-      <c r="N19" s="28"/>
-      <c r="O19" s="28"/>
+      <c r="L19" s="27"/>
+      <c r="M19" s="27"/>
+      <c r="N19" s="27"/>
+      <c r="O19" s="27"/>
     </row>
     <row r="20" spans="3:15" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C20" s="4"/>
@@ -2408,11 +2408,11 @@
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
-      <c r="K21" s="26"/>
-      <c r="L21" s="26"/>
-      <c r="M21" s="26"/>
-      <c r="N21" s="26"/>
-      <c r="O21" s="26"/>
+      <c r="K21" s="21"/>
+      <c r="L21" s="21"/>
+      <c r="M21" s="21"/>
+      <c r="N21" s="21"/>
+      <c r="O21" s="21"/>
     </row>
     <row r="22" spans="3:15" ht="57" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C22" s="4"/>
@@ -2420,14 +2420,14 @@
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
-      <c r="K22" s="29" t="str">
+      <c r="K22" s="28" t="str">
         <f>UPPER(student_name)</f>
         <v>PRINCE JONE ARMAN JOHN MARS C. DELA CRUZ</v>
       </c>
-      <c r="L22" s="29"/>
-      <c r="M22" s="29"/>
-      <c r="N22" s="29"/>
-      <c r="O22" s="29"/>
+      <c r="L22" s="28"/>
+      <c r="M22" s="28"/>
+      <c r="N22" s="28"/>
+      <c r="O22" s="28"/>
     </row>
     <row r="23" spans="3:15" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C23" s="4"/>
@@ -2435,11 +2435,11 @@
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
-      <c r="K23" s="26"/>
-      <c r="L23" s="26"/>
-      <c r="M23" s="26"/>
-      <c r="N23" s="26"/>
-      <c r="O23" s="26"/>
+      <c r="K23" s="21"/>
+      <c r="L23" s="21"/>
+      <c r="M23" s="21"/>
+      <c r="N23" s="21"/>
+      <c r="O23" s="21"/>
     </row>
     <row r="24" spans="3:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C24" s="4"/>
@@ -2447,7 +2447,7 @@
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
-      <c r="K24" s="30" t="str">
+      <c r="K24" s="26" t="str">
         <f t="array" ref="K24">_xlfn.LET(
  _xlpm.s,LOWER(TRIM(status)),
  _xlpm.prog,program,
@@ -2485,39 +2485,39 @@
 )</f>
         <v>was a student in this University enrolled in the Civil Engineering Technology program from 2015 to 2016.</v>
       </c>
-      <c r="L24" s="30"/>
-      <c r="M24" s="30"/>
-      <c r="N24" s="30"/>
-      <c r="O24" s="30"/>
+      <c r="L24" s="26"/>
+      <c r="M24" s="26"/>
+      <c r="N24" s="26"/>
+      <c r="O24" s="26"/>
     </row>
     <row r="25" spans="3:15" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
-      <c r="K25" s="30"/>
-      <c r="L25" s="30"/>
-      <c r="M25" s="30"/>
-      <c r="N25" s="30"/>
-      <c r="O25" s="30"/>
+      <c r="K25" s="26"/>
+      <c r="L25" s="26"/>
+      <c r="M25" s="26"/>
+      <c r="N25" s="26"/>
+      <c r="O25" s="26"/>
     </row>
     <row r="26" spans="3:15" ht="10.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D26" s="4"/>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
-      <c r="K26" s="31"/>
-      <c r="L26" s="31"/>
-      <c r="M26" s="31"/>
-      <c r="N26" s="31"/>
-      <c r="O26" s="31"/>
+      <c r="K26" s="23"/>
+      <c r="L26" s="23"/>
+      <c r="M26" s="23"/>
+      <c r="N26" s="23"/>
+      <c r="O26" s="23"/>
     </row>
     <row r="27" spans="3:15" ht="78" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D27" s="4"/>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
-      <c r="K27" s="30" t="str">
+      <c r="K27" s="26" t="str">
         <f>IF(LOWER(sex)="male","He",
    IF(LOWER(sex)="female","She","They")
  ) &amp;
@@ -2528,17 +2528,17 @@
  " stay in the University."</f>
         <v>He was a student of good moral standing, has no records of violating the school rules and regulations, and has not been subjected to any disciplinary action during his stay in the University.</v>
       </c>
-      <c r="L27" s="30"/>
-      <c r="M27" s="30"/>
-      <c r="N27" s="30"/>
-      <c r="O27" s="30"/>
+      <c r="L27" s="26"/>
+      <c r="M27" s="26"/>
+      <c r="N27" s="26"/>
+      <c r="O27" s="26"/>
     </row>
     <row r="28" spans="3:15" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D28" s="4"/>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
-      <c r="K28" s="30" t="str">
+      <c r="K28" s="26" t="str">
         <f ca="1">_xlfn.LET(_xlpm.d,DAY(TODAY()),
      _xlpm.suf,IF(OR(_xlpm.d=11,_xlpm.d=12,_xlpm.d=13),"th",
             CHOOSE(1+MOD(_xlpm.d,10),"th","st","nd","rd","th","th","th","th","th","th")),
@@ -2546,145 +2546,145 @@
  " at TUP Cavite Campus as a requirement for " &amp; purpose &amp; ".")</f>
         <v>Given this 19th day of November 2025 at TUP Cavite Campus as a requirement for continuing education.</v>
       </c>
-      <c r="L28" s="30"/>
-      <c r="M28" s="30"/>
-      <c r="N28" s="30"/>
-      <c r="O28" s="30"/>
+      <c r="L28" s="26"/>
+      <c r="M28" s="26"/>
+      <c r="N28" s="26"/>
+      <c r="O28" s="26"/>
     </row>
     <row r="29" spans="3:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D29" s="4"/>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
-      <c r="K29" s="31"/>
-      <c r="L29" s="31"/>
-      <c r="M29" s="31"/>
-      <c r="N29" s="31"/>
-      <c r="O29" s="31"/>
+      <c r="K29" s="23"/>
+      <c r="L29" s="23"/>
+      <c r="M29" s="23"/>
+      <c r="N29" s="23"/>
+      <c r="O29" s="23"/>
     </row>
     <row r="30" spans="3:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
-      <c r="K30" s="31"/>
-      <c r="L30" s="31"/>
-      <c r="M30" s="31"/>
-      <c r="N30" s="31"/>
-      <c r="O30" s="31"/>
+      <c r="K30" s="23"/>
+      <c r="L30" s="23"/>
+      <c r="M30" s="23"/>
+      <c r="N30" s="23"/>
+      <c r="O30" s="23"/>
     </row>
     <row r="31" spans="3:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
-      <c r="K31" s="31"/>
-      <c r="L31" s="31"/>
-      <c r="M31" s="31"/>
-      <c r="N31" s="31"/>
-      <c r="O31" s="31"/>
+      <c r="K31" s="23"/>
+      <c r="L31" s="23"/>
+      <c r="M31" s="23"/>
+      <c r="N31" s="23"/>
+      <c r="O31" s="23"/>
     </row>
     <row r="32" spans="3:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D32" s="4"/>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
-      <c r="K32" s="31"/>
-      <c r="L32" s="31"/>
-      <c r="M32" s="31"/>
-      <c r="N32" s="31"/>
-      <c r="O32" s="31"/>
+      <c r="K32" s="23"/>
+      <c r="L32" s="23"/>
+      <c r="M32" s="23"/>
+      <c r="N32" s="23"/>
+      <c r="O32" s="23"/>
     </row>
     <row r="33" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D33" s="4"/>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
-      <c r="K33" s="31"/>
-      <c r="L33" s="31"/>
-      <c r="M33" s="31"/>
-      <c r="N33" s="31"/>
-      <c r="O33" s="31"/>
+      <c r="K33" s="23"/>
+      <c r="L33" s="23"/>
+      <c r="M33" s="23"/>
+      <c r="N33" s="23"/>
+      <c r="O33" s="23"/>
     </row>
     <row r="34" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D34" s="4"/>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
-      <c r="K34" s="31"/>
-      <c r="L34" s="31"/>
-      <c r="M34" s="31"/>
-      <c r="N34" s="31"/>
-      <c r="O34" s="31"/>
+      <c r="K34" s="23"/>
+      <c r="L34" s="23"/>
+      <c r="M34" s="23"/>
+      <c r="N34" s="23"/>
+      <c r="O34" s="23"/>
     </row>
     <row r="35" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D35" s="4"/>
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
-      <c r="K35" s="31"/>
-      <c r="L35" s="31"/>
-      <c r="M35" s="31"/>
-      <c r="N35" s="31"/>
-      <c r="O35" s="31"/>
+      <c r="K35" s="23"/>
+      <c r="L35" s="23"/>
+      <c r="M35" s="23"/>
+      <c r="N35" s="23"/>
+      <c r="O35" s="23"/>
     </row>
     <row r="36" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
-      <c r="K36" s="32"/>
-      <c r="L36" s="32"/>
-      <c r="M36" s="32"/>
-      <c r="N36" s="32"/>
-      <c r="O36" s="32"/>
+      <c r="K36" s="22"/>
+      <c r="L36" s="22"/>
+      <c r="M36" s="22"/>
+      <c r="N36" s="22"/>
+      <c r="O36" s="22"/>
     </row>
     <row r="37" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
-      <c r="K37" s="31"/>
-      <c r="L37" s="31"/>
-      <c r="M37" s="31"/>
-      <c r="N37" s="31"/>
-      <c r="O37" s="31"/>
+      <c r="K37" s="23"/>
+      <c r="L37" s="23"/>
+      <c r="M37" s="23"/>
+      <c r="N37" s="23"/>
+      <c r="O37" s="23"/>
     </row>
     <row r="38" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
-      <c r="K38" s="26"/>
-      <c r="L38" s="26"/>
-      <c r="M38" s="26"/>
-      <c r="N38" s="26"/>
-      <c r="O38" s="26"/>
+      <c r="K38" s="21"/>
+      <c r="L38" s="21"/>
+      <c r="M38" s="21"/>
+      <c r="N38" s="21"/>
+      <c r="O38" s="21"/>
     </row>
     <row r="39" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
-      <c r="K39" s="32"/>
-      <c r="L39" s="32"/>
-      <c r="M39" s="32"/>
-      <c r="N39" s="32"/>
-      <c r="O39" s="32"/>
+      <c r="K39" s="22"/>
+      <c r="L39" s="22"/>
+      <c r="M39" s="22"/>
+      <c r="N39" s="22"/>
+      <c r="O39" s="22"/>
     </row>
     <row r="40" spans="4:15" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
-      <c r="K40" s="32" t="str">
+      <c r="K40" s="22" t="str">
         <f t="array" ref="K40">UPPER(osahead)</f>
         <v>BEVERLY M. DE VEGA</v>
       </c>
-      <c r="L40" s="32"/>
-      <c r="M40" s="32"/>
-      <c r="N40" s="32"/>
-      <c r="O40" s="32"/>
+      <c r="L40" s="22"/>
+      <c r="M40" s="22"/>
+      <c r="N40" s="22"/>
+      <c r="O40" s="22"/>
     </row>
     <row r="41" spans="4:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D41" s="4"/>
@@ -2692,80 +2692,80 @@
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="13"/>
-      <c r="K41" s="33" t="str">
-        <f>title</f>
+      <c r="K41" s="24" t="str">
+        <f>osahead_title</f>
         <v>Head, Office of Student Affairs</v>
       </c>
-      <c r="L41" s="34"/>
-      <c r="M41" s="34"/>
-      <c r="N41" s="34"/>
-      <c r="O41" s="34"/>
+      <c r="L41" s="25"/>
+      <c r="M41" s="25"/>
+      <c r="N41" s="25"/>
+      <c r="O41" s="25"/>
     </row>
     <row r="42" spans="4:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
-      <c r="K42" s="26"/>
-      <c r="L42" s="26"/>
-      <c r="M42" s="26"/>
-      <c r="N42" s="26"/>
-      <c r="O42" s="26"/>
+      <c r="K42" s="21"/>
+      <c r="L42" s="21"/>
+      <c r="M42" s="21"/>
+      <c r="N42" s="21"/>
+      <c r="O42" s="21"/>
     </row>
     <row r="43" spans="4:15" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
-      <c r="K43" s="26"/>
-      <c r="L43" s="26"/>
-      <c r="M43" s="26"/>
-      <c r="N43" s="26"/>
-      <c r="O43" s="26"/>
+      <c r="K43" s="21"/>
+      <c r="L43" s="21"/>
+      <c r="M43" s="21"/>
+      <c r="N43" s="21"/>
+      <c r="O43" s="21"/>
     </row>
     <row r="44" spans="4:15" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D44" s="4"/>
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
-      <c r="K44" s="26"/>
-      <c r="L44" s="26"/>
-      <c r="M44" s="26"/>
-      <c r="N44" s="26"/>
-      <c r="O44" s="26"/>
+      <c r="K44" s="21"/>
+      <c r="L44" s="21"/>
+      <c r="M44" s="21"/>
+      <c r="N44" s="21"/>
+      <c r="O44" s="21"/>
     </row>
     <row r="45" spans="4:15" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D45" s="4"/>
       <c r="E45" s="4"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
-      <c r="K45" s="26"/>
-      <c r="L45" s="26"/>
-      <c r="M45" s="26"/>
-      <c r="N45" s="26"/>
-      <c r="O45" s="26"/>
+      <c r="K45" s="21"/>
+      <c r="L45" s="21"/>
+      <c r="M45" s="21"/>
+      <c r="N45" s="21"/>
+      <c r="O45" s="21"/>
     </row>
     <row r="46" spans="4:15" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D46" s="4"/>
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
-      <c r="K46" s="26"/>
-      <c r="L46" s="26"/>
-      <c r="M46" s="26"/>
-      <c r="N46" s="26"/>
-      <c r="O46" s="26"/>
+      <c r="K46" s="21"/>
+      <c r="L46" s="21"/>
+      <c r="M46" s="21"/>
+      <c r="N46" s="21"/>
+      <c r="O46" s="21"/>
     </row>
     <row r="47" spans="4:15" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D47" s="4"/>
       <c r="E47" s="4"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
-      <c r="K47" s="26"/>
-      <c r="L47" s="26"/>
-      <c r="M47" s="26"/>
-      <c r="N47" s="26"/>
-      <c r="O47" s="26"/>
+      <c r="K47" s="21"/>
+      <c r="L47" s="21"/>
+      <c r="M47" s="21"/>
+      <c r="N47" s="21"/>
+      <c r="O47" s="21"/>
     </row>
     <row r="48" spans="4:15" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D48" s="4"/>
@@ -8520,11 +8520,31 @@
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="K42:O42"/>
-    <mergeCell ref="K43:O43"/>
-    <mergeCell ref="K44:O44"/>
-    <mergeCell ref="K45:O45"/>
-    <mergeCell ref="K46:O46"/>
+    <mergeCell ref="H2:P2"/>
+    <mergeCell ref="H5:P5"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="H6:P6"/>
+    <mergeCell ref="H7:P7"/>
+    <mergeCell ref="H9:P9"/>
+    <mergeCell ref="K13:O13"/>
+    <mergeCell ref="K15:O15"/>
+    <mergeCell ref="K17:O17"/>
+    <mergeCell ref="K18:O18"/>
+    <mergeCell ref="K19:O19"/>
+    <mergeCell ref="K21:O21"/>
+    <mergeCell ref="K22:O22"/>
+    <mergeCell ref="K23:O23"/>
+    <mergeCell ref="K24:O25"/>
+    <mergeCell ref="K26:O26"/>
+    <mergeCell ref="K27:O27"/>
+    <mergeCell ref="K28:O28"/>
+    <mergeCell ref="K29:O29"/>
+    <mergeCell ref="K30:O30"/>
+    <mergeCell ref="K31:O31"/>
+    <mergeCell ref="K32:O32"/>
+    <mergeCell ref="K33:O33"/>
+    <mergeCell ref="K34:O34"/>
+    <mergeCell ref="K35:O35"/>
     <mergeCell ref="K47:O47"/>
     <mergeCell ref="K36:O36"/>
     <mergeCell ref="K37:O37"/>
@@ -8532,31 +8552,11 @@
     <mergeCell ref="K39:O39"/>
     <mergeCell ref="K40:O40"/>
     <mergeCell ref="K41:O41"/>
-    <mergeCell ref="K31:O31"/>
-    <mergeCell ref="K32:O32"/>
-    <mergeCell ref="K33:O33"/>
-    <mergeCell ref="K34:O34"/>
-    <mergeCell ref="K35:O35"/>
-    <mergeCell ref="K26:O26"/>
-    <mergeCell ref="K27:O27"/>
-    <mergeCell ref="K28:O28"/>
-    <mergeCell ref="K29:O29"/>
-    <mergeCell ref="K30:O30"/>
-    <mergeCell ref="K19:O19"/>
-    <mergeCell ref="K21:O21"/>
-    <mergeCell ref="K22:O22"/>
-    <mergeCell ref="K23:O23"/>
-    <mergeCell ref="K24:O25"/>
-    <mergeCell ref="H9:P9"/>
-    <mergeCell ref="K13:O13"/>
-    <mergeCell ref="K15:O15"/>
-    <mergeCell ref="K17:O17"/>
-    <mergeCell ref="K18:O18"/>
-    <mergeCell ref="H2:P2"/>
-    <mergeCell ref="H5:P5"/>
-    <mergeCell ref="D6:G6"/>
-    <mergeCell ref="H6:P6"/>
-    <mergeCell ref="H7:P7"/>
+    <mergeCell ref="K42:O42"/>
+    <mergeCell ref="K43:O43"/>
+    <mergeCell ref="K44:O44"/>
+    <mergeCell ref="K45:O45"/>
+    <mergeCell ref="K46:O46"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D6" xr:uid="{00000000-0002-0000-0100-000000000000}">

</xml_diff>